<commit_message>
Update user manager, requirements, gitignore
</commit_message>
<xml_diff>
--- a/Users.xlsx
+++ b/Users.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENTHILKUMARAN\Documents\My Codzz\000 Final Year Project\Sample 009\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENTHILKUMARAN\Documents\My Codzz\000 Final Year Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8200BFA-2634-4118-A8C8-7A981AF742A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDD7DFB-AD9C-4D2E-A975-68CBDAC2B6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A208323D-8702-4339-9656-4FCAD6907B9E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A208323D-8702-4339-9656-4FCAD6907B9E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="User's" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
-  <si>
-    <t>SI.No</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>Name</t>
   </si>
@@ -95,12 +92,6 @@
     <t>mani@gmail.com</t>
   </si>
   <si>
-    <t>Murugesan</t>
-  </si>
-  <si>
-    <t>mru@gmail.com</t>
-  </si>
-  <si>
     <t>jk@gmail.com</t>
   </si>
   <si>
@@ -116,15 +107,6 @@
     <t>kum@gamil.com</t>
   </si>
   <si>
-    <t>Vadivel</t>
-  </si>
-  <si>
-    <t>vadi@gmail.com</t>
-  </si>
-  <si>
-    <t>occupation</t>
-  </si>
-  <si>
     <t>Software Engineer</t>
   </si>
   <si>
@@ -159,13 +141,151 @@
   </si>
   <si>
     <t>IPS</t>
+  </si>
+  <si>
+    <t>Hari</t>
+  </si>
+  <si>
+    <t>hari@gmail.com</t>
+  </si>
+  <si>
+    <t>Magudesh</t>
+  </si>
+  <si>
+    <t>magu@gmail.com</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Salem</t>
+  </si>
+  <si>
+    <t>Erode</t>
+  </si>
+  <si>
+    <t>Theni</t>
+  </si>
+  <si>
+    <t>Omalur</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Edapadi</t>
+  </si>
+  <si>
+    <t>Ambur</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Sangagari</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
+  </si>
+  <si>
+    <t>Rasipuram</t>
+  </si>
+  <si>
+    <t>Karur</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t>Bank Name</t>
+  </si>
+  <si>
+    <t>Account Type</t>
+  </si>
+  <si>
+    <t>Bank Location</t>
+  </si>
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>Occupation</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>Senthilkumaran@123</t>
+  </si>
+  <si>
+    <t>Imayavarman@123</t>
+  </si>
+  <si>
+    <t>Srivarshan@123</t>
+  </si>
+  <si>
+    <t>Rahulprasath@123</t>
+  </si>
+  <si>
+    <t>Magudesh@123</t>
+  </si>
+  <si>
+    <t>Deepak@123</t>
+  </si>
+  <si>
+    <t>Mani@123</t>
+  </si>
+  <si>
+    <t>Dineshkumar@123</t>
+  </si>
+  <si>
+    <t>Avinash@123</t>
+  </si>
+  <si>
+    <t>Kumar@123</t>
+  </si>
+  <si>
+    <t>Hari@123</t>
+  </si>
+  <si>
+    <t>Janakrishnan@123</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Indian</t>
+  </si>
+  <si>
+    <t>KVB</t>
+  </si>
+  <si>
+    <t>Canara</t>
+  </si>
+  <si>
+    <t>AXIS</t>
+  </si>
+  <si>
+    <t>SBI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,8 +303,34 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Consolas"/>
-      <family val="3"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -208,15 +354,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -553,274 +714,555 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48537B8A-FD06-414F-B4BC-BF02FA4E6915}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.85546875" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" customWidth="1"/>
+    <col min="11" max="11" width="21.85546875" customWidth="1"/>
+    <col min="12" max="12" width="8" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="C2" s="11">
+        <v>22243045</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1010101010</v>
+      </c>
+      <c r="G2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="2">
+        <v>24</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="10">
+        <v>22243017</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1111111111</v>
+      </c>
+      <c r="G3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" t="s">
+        <v>74</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="2">
+        <v>32</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10">
+        <v>22243050</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1212121212</v>
+      </c>
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" t="s">
+        <v>74</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="2">
+        <v>40</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="10">
+        <v>22243040</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1313131313</v>
+      </c>
+      <c r="G5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" s="2">
+        <v>30</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="10">
+        <v>22243055</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1414141414</v>
+      </c>
+      <c r="G6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="2">
         <v>28</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>39</v>
+      <c r="M6" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="10">
+        <v>22243009</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="2">
+        <v>2020202020</v>
+      </c>
+      <c r="G7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L7" s="2">
+        <v>29</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="10">
+        <v>22243060</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="2">
+        <v>2121212121</v>
+      </c>
+      <c r="G8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="2">
+        <v>38</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="10">
+        <v>22243012</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2222222222</v>
+      </c>
+      <c r="G9" t="s">
+        <v>76</v>
+      </c>
+      <c r="H9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L9" s="2">
+        <v>52</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="10">
+        <v>22243007</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="2">
+        <v>2525252525</v>
+      </c>
+      <c r="G10" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J10" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="2">
+        <v>28</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="10">
+        <v>22243020</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="2">
+        <v>3333333333</v>
+      </c>
+      <c r="G11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L11" s="2">
+        <v>23</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="10">
+        <v>22243016</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="2">
+        <v>4444444444</v>
+      </c>
+      <c r="G12" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J12" t="s">
+        <v>74</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="L12" s="2">
+        <v>44</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
-        <v>1010101010</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="C13" s="10">
+        <v>22243019</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" s="2">
+        <v>5555555555</v>
+      </c>
+      <c r="G13" t="s">
+        <v>80</v>
+      </c>
+      <c r="H13" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F2">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3">
-        <v>1111111111</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>1212121212</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5">
-        <v>1313131313</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6">
-        <v>1414141414</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7">
-        <v>2020202020</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8">
-        <v>2121212121</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9">
-        <v>2222222222</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="L13" s="2">
         <v>22</v>
       </c>
-      <c r="C10">
-        <v>2525252525</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F10">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11">
-        <v>3333333333</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12">
-        <v>4444444444</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13">
-        <v>5555555555</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13">
-        <v>22</v>
+      <c r="M13" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -837,8 +1279,20 @@
     <hyperlink ref="D10" r:id="rId10" xr:uid="{DB4DBBFD-9EC9-472F-8FF6-77992D67DD7E}"/>
     <hyperlink ref="D11" r:id="rId11" xr:uid="{5977137B-FC48-453A-B8BA-EE95A7631015}"/>
     <hyperlink ref="D12" r:id="rId12" xr:uid="{BFA6D605-97F7-47E1-BC84-D54132C98D2F}"/>
+    <hyperlink ref="E2" r:id="rId13" xr:uid="{9B4E5D62-0C20-4F86-8319-6E558B0E2290}"/>
+    <hyperlink ref="E3" r:id="rId14" xr:uid="{36009235-F544-4752-BE0E-8057DEB7EF91}"/>
+    <hyperlink ref="E4" r:id="rId15" xr:uid="{048EE87C-EFBD-4F4D-90ED-1382D6BF5584}"/>
+    <hyperlink ref="E5" r:id="rId16" xr:uid="{D75B5A7D-3A5C-4D3B-A3A0-6ED94FC9A4E3}"/>
+    <hyperlink ref="E6" r:id="rId17" xr:uid="{0BF39D51-C20B-4852-9AF4-ABF7A299D033}"/>
+    <hyperlink ref="E7" r:id="rId18" xr:uid="{D54D741D-D76A-4685-848B-38235CD314BA}"/>
+    <hyperlink ref="E8" r:id="rId19" xr:uid="{3DAAEB23-E2A5-4E6D-BCA7-2DBD684A4F82}"/>
+    <hyperlink ref="E9" r:id="rId20" xr:uid="{1222B3D8-C97F-4F6E-8653-A85DFAA94CF6}"/>
+    <hyperlink ref="E10" r:id="rId21" xr:uid="{03AA8975-6C1F-474D-ACF5-41FF1139B0D6}"/>
+    <hyperlink ref="E11" r:id="rId22" xr:uid="{84B35E2A-D7C8-4E8B-B493-6DFA2727E762}"/>
+    <hyperlink ref="E12" r:id="rId23" xr:uid="{D70823C6-371B-45B3-A239-3947115B7234}"/>
+    <hyperlink ref="E13" r:id="rId24" xr:uid="{518C037F-F06C-48FF-9464-A53727E3DD1D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId13"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>